<commit_message>
Addition of PMM Module by Grassroots in collaboration with WHO & Path
</commit_message>
<xml_diff>
--- a/app/config/tables/maintenance_logs/forms/maintenance_logs/maintenance_logs.xlsx
+++ b/app/config/tables/maintenance_logs/forms/maintenance_logs/maintenance_logs.xlsx
@@ -1,30 +1,32 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\clarice\cold-chain\cold-chain-app-designer\app\config\tables\maintenance_logs\forms\maintenance_logs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Projects\ODK-X\our-work\app\config\tables\maintenance_logs\forms\maintenance_logs\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A30B0785-9EAA-413B-B9A1-FC1DC315E90D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11060" yWindow="2690" windowWidth="28370" windowHeight="19560" tabRatio="500" activeTab="1"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="initial" sheetId="6" r:id="rId1"/>
     <sheet name="survey" sheetId="1" r:id="rId2"/>
-    <sheet name="choices" sheetId="2" r:id="rId3"/>
-    <sheet name="queries" sheetId="3" r:id="rId4"/>
-    <sheet name="settings" sheetId="4" r:id="rId5"/>
-    <sheet name="properties" sheetId="5" r:id="rId6"/>
+    <sheet name="model" sheetId="7" r:id="rId3"/>
+    <sheet name="choices" sheetId="2" r:id="rId4"/>
+    <sheet name="queries" sheetId="3" r:id="rId5"/>
+    <sheet name="settings" sheetId="4" r:id="rId6"/>
+    <sheet name="properties" sheetId="5" r:id="rId7"/>
   </sheets>
   <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="659" uniqueCount="476">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="684" uniqueCount="484">
   <si>
     <t>clause</t>
   </si>
@@ -1453,12 +1455,36 @@
   </si>
   <si>
     <t>Acciones tomadas</t>
+  </si>
+  <si>
+    <t>under_warranty = ?</t>
+  </si>
+  <si>
+    <t>['yes']</t>
+  </si>
+  <si>
+    <t>under_warranty</t>
+  </si>
+  <si>
+    <t>isSessionVariable</t>
+  </si>
+  <si>
+    <t>warranty_service_provider_name</t>
+  </si>
+  <si>
+    <t>warranty_service_provider_contact</t>
+  </si>
+  <si>
+    <t>data('under_warranty') === 'yes'</t>
+  </si>
+  <si>
+    <t>&lt;p style="color: red;"&gt;This device is currently under warranty, for repairs contact [{{data.warranty_service_provider_contact}}], be sure to update refrigerator status and notes.&lt;/p&gt;</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -1619,30 +1645,26 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1651,41 +1673,19 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="40" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="40" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1730,7 +1730,7 @@
     <cellStyle name="Hyperlink" xfId="36" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="38" builtinId="8" hidden="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="40"/>
+    <cellStyle name="Normal 2" xfId="40" xr:uid="{00000000-0005-0000-0000-000028000000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
@@ -2134,15 +2134,13 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D3"/>
   <sheetFormatPr defaultColWidth="8.75" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16" style="28" customWidth="1"/>
-    <col min="2" max="2" width="8.75" style="28"/>
-    <col min="3" max="3" width="18" style="28" customWidth="1"/>
-    <col min="4" max="4" width="24.25" style="28" customWidth="1"/>
-    <col min="5" max="16384" width="8.75" style="28"/>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="24.25" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
@@ -2183,12 +2181,12 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L40"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:L43"/>
   <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="2" max="2" width="43.1640625" style="1" customWidth="1"/>
     <col min="3" max="3" width="20" customWidth="1"/>
     <col min="4" max="4" width="26.08203125" customWidth="1"/>
     <col min="5" max="5" width="25.08203125" customWidth="1"/>
@@ -2231,7 +2229,7 @@
       <c r="J1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="K1" s="22" t="s">
+      <c r="K1" s="1" t="s">
         <v>347</v>
       </c>
       <c r="L1" t="s">
@@ -2242,7 +2240,6 @@
       <c r="A2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="1"/>
       <c r="C2" s="1"/>
       <c r="D2" s="2"/>
       <c r="E2" s="1"/>
@@ -2251,13 +2248,13 @@
       <c r="H2" s="1"/>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
-      <c r="K2" s="22"/>
+      <c r="K2" s="1"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="1">
         <v>0</v>
       </c>
       <c r="C3" s="1"/>
@@ -2268,11 +2265,10 @@
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
-      <c r="K3" s="22"/>
+      <c r="K3" s="1"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A4" s="1"/>
-      <c r="B4" s="1"/>
       <c r="C4" s="1" t="s">
         <v>12</v>
       </c>
@@ -2292,7 +2288,7 @@
       <c r="J4" t="s">
         <v>17</v>
       </c>
-      <c r="K4" s="21" t="s">
+      <c r="K4" t="s">
         <v>365</v>
       </c>
       <c r="L4">
@@ -2300,630 +2296,651 @@
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
+      <c r="A5" s="1" t="s">
         <v>18</v>
       </c>
       <c r="C5" s="1"/>
       <c r="D5" s="2"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
-      <c r="G5" s="1"/>
-      <c r="H5" s="1"/>
-      <c r="I5" s="1"/>
-      <c r="J5" s="1"/>
-      <c r="K5" s="22"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1" t="s">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="124" x14ac:dyDescent="0.35">
+      <c r="C7" t="s">
+        <v>397</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>483</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F8" s="1"/>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A9" s="1"/>
+      <c r="C9" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E9" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="F9" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="G9" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="H6" s="1"/>
-      <c r="I6" s="1" t="s">
+      <c r="H9" s="1"/>
+      <c r="I9" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="J6" s="14" t="s">
+      <c r="J9" s="12" t="s">
         <v>135</v>
       </c>
-      <c r="K6" s="22" t="s">
+      <c r="K9" s="1" t="s">
         <v>366</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1" t="s">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A10" s="1"/>
+      <c r="C10" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="D7" s="2"/>
-      <c r="E7" s="1" t="s">
+      <c r="D10" s="2"/>
+      <c r="E10" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="F7" s="1" t="s">
+      <c r="F10" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="G10" s="1" t="s">
         <v>137</v>
       </c>
-      <c r="H7" s="1"/>
-      <c r="I7" s="1" t="s">
+      <c r="H10" s="1"/>
+      <c r="I10" s="1" t="s">
         <v>139</v>
       </c>
-      <c r="J7" s="1" t="s">
+      <c r="J10" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="K7" s="22" t="s">
+      <c r="K10" s="1" t="s">
         <v>367</v>
       </c>
     </row>
-    <row r="8" spans="1:12" s="30" customFormat="1" ht="31" x14ac:dyDescent="0.35">
-      <c r="A8" s="32"/>
-      <c r="B8" s="32"/>
-      <c r="C8" s="32" t="s">
+    <row r="11" spans="1:12" s="15" customFormat="1" ht="31" x14ac:dyDescent="0.35">
+      <c r="A11" s="16"/>
+      <c r="B11" s="16"/>
+      <c r="C11" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="D8" s="33"/>
-      <c r="E8" s="32" t="s">
+      <c r="D11" s="17"/>
+      <c r="E11" s="16" t="s">
         <v>388</v>
       </c>
-      <c r="F8" s="32" t="s">
+      <c r="F11" s="16" t="s">
         <v>389</v>
       </c>
-      <c r="G8" s="32" t="s">
+      <c r="G11" s="16" t="s">
         <v>398</v>
       </c>
-      <c r="H8" s="32"/>
-      <c r="I8" s="32" t="s">
+      <c r="H11" s="16"/>
+      <c r="I11" s="16" t="s">
         <v>399</v>
       </c>
-      <c r="J8" s="32" t="s">
+      <c r="J11" s="16" t="s">
         <v>400</v>
       </c>
-      <c r="K8" s="32"/>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A9" s="1" t="s">
+      <c r="K11" s="16"/>
+    </row>
+    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A12" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="1"/>
-      <c r="F9" s="1"/>
-      <c r="G9" s="1"/>
-      <c r="H9" s="1"/>
-      <c r="I9" s="1"/>
-      <c r="J9" s="1"/>
-      <c r="K9" s="22"/>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="A10" s="1" t="s">
+      <c r="C12" s="1"/>
+      <c r="D12" s="2"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
+      <c r="G12" s="1"/>
+      <c r="H12" s="1"/>
+      <c r="I12" s="1"/>
+      <c r="J12" s="1"/>
+      <c r="K12" s="1"/>
+    </row>
+    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="A13" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="1"/>
-      <c r="F10" s="1"/>
-      <c r="G10" s="1"/>
-      <c r="H10" s="1"/>
-      <c r="I10" s="1"/>
-      <c r="J10" s="1"/>
-      <c r="K10" s="22"/>
-    </row>
-    <row r="11" spans="1:12" s="30" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="C11" s="31" t="s">
+      <c r="C13" s="1"/>
+      <c r="D13" s="2"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
+      <c r="G13" s="1"/>
+      <c r="H13" s="1"/>
+      <c r="I13" s="1"/>
+      <c r="J13" s="1"/>
+      <c r="K13" s="1"/>
+    </row>
+    <row r="14" spans="1:12" s="15" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B14" s="16"/>
+      <c r="C14" s="15" t="s">
         <v>345</v>
       </c>
-      <c r="D11" s="31"/>
-      <c r="E11" s="31" t="s">
+      <c r="E14" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="F11" s="31" t="s">
+      <c r="F14" s="15" t="s">
         <v>384</v>
       </c>
-      <c r="G11" s="31" t="s">
+      <c r="G14" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="H11" s="31"/>
-      <c r="I11" s="31" t="s">
+      <c r="I14" s="15" t="s">
         <v>385</v>
       </c>
-      <c r="J11" s="30" t="s">
+      <c r="J14" s="15" t="s">
         <v>386</v>
       </c>
-      <c r="K11" s="32" t="s">
+      <c r="K14" s="16" t="s">
         <v>387</v>
       </c>
     </row>
-    <row r="12" spans="1:12" s="30" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="C12" s="32" t="s">
+    <row r="15" spans="1:12" s="15" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B15" s="16"/>
+      <c r="C15" s="16" t="s">
         <v>390</v>
       </c>
-      <c r="E12" s="30" t="s">
+      <c r="E15" s="15" t="s">
         <v>473</v>
       </c>
-      <c r="F12" s="30" t="s">
+      <c r="F15" s="15" t="s">
         <v>474</v>
       </c>
-      <c r="G12" s="30" t="s">
+      <c r="G15" s="15" t="s">
         <v>475</v>
       </c>
-      <c r="I12" s="30" t="s">
+      <c r="I15" s="15" t="s">
         <v>426</v>
       </c>
-      <c r="J12" s="34" t="s">
+      <c r="J15" s="16" t="s">
         <v>427</v>
       </c>
-      <c r="K12" s="32"/>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
-      <c r="C13" s="1" t="s">
+      <c r="K15" s="16"/>
+    </row>
+    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
+      <c r="C16" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D16" t="s">
         <v>82</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E16" t="s">
         <v>79</v>
       </c>
-      <c r="F13" t="s">
+      <c r="F16" t="s">
         <v>80</v>
       </c>
-      <c r="G13" t="s">
+      <c r="G16" t="s">
         <v>81</v>
       </c>
-      <c r="I13" t="s">
+      <c r="I16" t="s">
         <v>92</v>
       </c>
-      <c r="J13" s="9" t="s">
+      <c r="J16" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="K13" s="22" t="s">
+      <c r="K16" s="1" t="s">
         <v>369</v>
       </c>
-    </row>
-    <row r="14" spans="1:12" s="28" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="28" t="s">
-        <v>11</v>
-      </c>
-      <c r="B14" s="28" t="s">
-        <v>428</v>
-      </c>
-      <c r="C14" s="1"/>
-      <c r="J14" s="9"/>
-      <c r="K14" s="22"/>
-    </row>
-    <row r="15" spans="1:12" s="30" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="C15" s="32" t="s">
-        <v>390</v>
-      </c>
-      <c r="E15" s="30" t="s">
-        <v>456</v>
-      </c>
-      <c r="F15" s="30" t="s">
-        <v>462</v>
-      </c>
-      <c r="G15" s="30" t="s">
-        <v>464</v>
-      </c>
-      <c r="I15" s="30" t="s">
-        <v>457</v>
-      </c>
-      <c r="J15" s="34" t="s">
-        <v>465</v>
-      </c>
-      <c r="K15" s="32"/>
-    </row>
-    <row r="16" spans="1:12" s="28" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="28" t="s">
-        <v>18</v>
-      </c>
-      <c r="C16" s="1"/>
-      <c r="J16" s="9"/>
-      <c r="K16" s="22"/>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>11</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="1" t="s">
+        <v>428</v>
+      </c>
+      <c r="C17" s="1"/>
+      <c r="J17" s="1"/>
+      <c r="K17" s="1"/>
+    </row>
+    <row r="18" spans="1:11" s="15" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B18" s="16"/>
+      <c r="C18" s="16" t="s">
+        <v>390</v>
+      </c>
+      <c r="E18" s="15" t="s">
+        <v>456</v>
+      </c>
+      <c r="F18" s="15" t="s">
+        <v>462</v>
+      </c>
+      <c r="G18" s="15" t="s">
+        <v>464</v>
+      </c>
+      <c r="I18" s="15" t="s">
+        <v>457</v>
+      </c>
+      <c r="J18" s="16" t="s">
+        <v>465</v>
+      </c>
+      <c r="K18" s="16"/>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>18</v>
+      </c>
+      <c r="C19" s="1"/>
+      <c r="J19" s="1"/>
+      <c r="K19" s="1"/>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>11</v>
+      </c>
+      <c r="B20" s="1" t="s">
         <v>451</v>
       </c>
-      <c r="C17" s="1"/>
-      <c r="J17" s="9"/>
-      <c r="K17" s="20"/>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="C18" s="1" t="s">
+      <c r="C20" s="1"/>
+      <c r="J20" s="1"/>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="C21" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="D18" t="s">
+      <c r="D21" t="s">
         <v>126</v>
       </c>
-      <c r="E18" t="s">
+      <c r="E21" t="s">
         <v>127</v>
       </c>
-      <c r="F18" t="s">
+      <c r="F21" t="s">
         <v>128</v>
       </c>
-      <c r="G18" t="s">
+      <c r="G21" t="s">
         <v>159</v>
       </c>
-      <c r="I18" t="s">
+      <c r="I21" t="s">
         <v>161</v>
       </c>
-      <c r="J18" s="9" t="s">
+      <c r="J21" s="1" t="s">
         <v>162</v>
       </c>
-      <c r="K18" s="22" t="s">
+      <c r="K21" s="1" t="s">
         <v>370</v>
       </c>
     </row>
-    <row r="19" spans="1:11" s="28" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="28" t="s">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A22" t="s">
         <v>11</v>
       </c>
-      <c r="B19" s="28" t="s">
+      <c r="B22" s="1" t="s">
         <v>425</v>
       </c>
-      <c r="C19" s="1"/>
-      <c r="J19" s="9"/>
-      <c r="K19" s="22"/>
-    </row>
-    <row r="20" spans="1:11" s="30" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="C20" s="32" t="s">
+      <c r="C22" s="1"/>
+      <c r="J22" s="1"/>
+      <c r="K22" s="1"/>
+    </row>
+    <row r="23" spans="1:11" s="15" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B23" s="16"/>
+      <c r="C23" s="16" t="s">
         <v>390</v>
       </c>
-      <c r="E20" s="30" t="s">
+      <c r="E23" s="15" t="s">
         <v>458</v>
       </c>
-      <c r="F20" s="30" t="s">
+      <c r="F23" s="15" t="s">
         <v>463</v>
       </c>
-      <c r="G20" s="30" t="s">
+      <c r="G23" s="15" t="s">
         <v>466</v>
       </c>
-      <c r="I20" s="30" t="s">
+      <c r="I23" s="15" t="s">
         <v>467</v>
       </c>
-      <c r="J20" s="34" t="s">
+      <c r="J23" s="16" t="s">
         <v>468</v>
       </c>
-      <c r="K20" s="32"/>
-    </row>
-    <row r="21" spans="1:11" s="28" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="28" t="s">
-        <v>18</v>
-      </c>
-      <c r="C21" s="1"/>
-      <c r="J21" s="9"/>
-      <c r="K21" s="22"/>
-    </row>
-    <row r="22" spans="1:11" s="30" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C22" s="30" t="s">
-        <v>12</v>
-      </c>
-      <c r="E22" s="30" t="s">
-        <v>460</v>
-      </c>
-      <c r="F22" s="30" t="s">
-        <v>461</v>
-      </c>
-      <c r="G22" s="30" t="s">
-        <v>469</v>
-      </c>
-      <c r="I22" s="30" t="s">
-        <v>459</v>
-      </c>
-      <c r="J22" s="30" t="s">
-        <v>470</v>
-      </c>
-      <c r="K22" s="32" t="s">
-        <v>368</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
-        <v>18</v>
-      </c>
-      <c r="C23" s="1"/>
-      <c r="J23" s="9"/>
-      <c r="K23" s="20"/>
+      <c r="K23" s="16"/>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
+        <v>18</v>
+      </c>
+      <c r="C24" s="1"/>
+      <c r="J24" s="1"/>
+      <c r="K24" s="1"/>
+    </row>
+    <row r="25" spans="1:11" s="15" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B25" s="16"/>
+      <c r="C25" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="E25" s="15" t="s">
+        <v>460</v>
+      </c>
+      <c r="F25" s="15" t="s">
+        <v>461</v>
+      </c>
+      <c r="G25" s="15" t="s">
+        <v>469</v>
+      </c>
+      <c r="I25" s="15" t="s">
+        <v>459</v>
+      </c>
+      <c r="J25" s="15" t="s">
+        <v>470</v>
+      </c>
+      <c r="K25" s="16" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
+        <v>18</v>
+      </c>
+      <c r="C26" s="1"/>
+      <c r="J26" s="1"/>
+    </row>
+    <row r="27" spans="1:11" ht="31" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
         <v>11</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B27" s="1" t="s">
         <v>434</v>
       </c>
-      <c r="C24" s="1"/>
-      <c r="J24" s="9"/>
-      <c r="K24" s="20"/>
-    </row>
-    <row r="25" spans="1:11" s="30" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="C25" s="32" t="s">
+      <c r="C27" s="1"/>
+      <c r="J27" s="1"/>
+    </row>
+    <row r="28" spans="1:11" s="15" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B28" s="16"/>
+      <c r="C28" s="16" t="s">
         <v>125</v>
       </c>
-      <c r="D25" s="30" t="s">
+      <c r="D28" s="15" t="s">
         <v>129</v>
       </c>
-      <c r="E25" s="30" t="s">
+      <c r="E28" s="15" t="s">
         <v>130</v>
       </c>
-      <c r="F25" s="30" t="s">
+      <c r="F28" s="15" t="s">
         <v>131</v>
       </c>
-      <c r="G25" s="30" t="s">
+      <c r="G28" s="15" t="s">
         <v>160</v>
       </c>
-      <c r="I25" s="30" t="s">
+      <c r="I28" s="15" t="s">
         <v>435</v>
       </c>
-      <c r="J25" s="34" t="s">
+      <c r="J28" s="16" t="s">
         <v>436</v>
       </c>
-      <c r="K25" s="34" t="s">
+      <c r="K28" s="16" t="s">
         <v>369</v>
       </c>
     </row>
-    <row r="26" spans="1:11" s="30" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="C26" s="32" t="s">
+    <row r="29" spans="1:11" s="15" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B29" s="16"/>
+      <c r="C29" s="16" t="s">
         <v>390</v>
       </c>
-      <c r="E26" s="30" t="s">
+      <c r="E29" s="15" t="s">
         <v>454</v>
       </c>
-      <c r="F26" s="30" t="s">
+      <c r="F29" s="15" t="s">
         <v>453</v>
       </c>
-      <c r="G26" s="30" t="s">
+      <c r="G29" s="15" t="s">
         <v>471</v>
       </c>
-      <c r="I26" s="30" t="s">
+      <c r="I29" s="15" t="s">
         <v>455</v>
       </c>
-      <c r="J26" s="34" t="s">
+      <c r="J29" s="16" t="s">
         <v>472</v>
       </c>
-      <c r="K26" s="34"/>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
-        <v>18</v>
-      </c>
-      <c r="C27" s="1"/>
-      <c r="J27" s="9"/>
-      <c r="K27" s="20"/>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A28" t="s">
-        <v>21</v>
-      </c>
-      <c r="C28" s="1"/>
-      <c r="J28" s="9"/>
-      <c r="K28" s="20"/>
-    </row>
-    <row r="29" spans="1:11" s="28" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="28" t="s">
-        <v>11</v>
-      </c>
-      <c r="B29" s="28" t="s">
-        <v>452</v>
-      </c>
-      <c r="C29" s="1"/>
-      <c r="J29" s="9"/>
+      <c r="K29" s="16"/>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
+        <v>18</v>
+      </c>
+      <c r="C30" s="1"/>
+      <c r="J30" s="1"/>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>21</v>
+      </c>
+      <c r="C31" s="1"/>
+      <c r="J31" s="1"/>
+    </row>
+    <row r="32" spans="1:11" ht="31" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>11</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>452</v>
+      </c>
+      <c r="C32" s="1"/>
+      <c r="J32" s="1"/>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
         <v>10</v>
       </c>
-      <c r="C30" s="1"/>
-      <c r="J30" s="9"/>
-      <c r="K30" s="20"/>
-    </row>
-    <row r="31" spans="1:11" s="30" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C31" s="32" t="s">
+      <c r="C33" s="1"/>
+      <c r="J33" s="1"/>
+    </row>
+    <row r="34" spans="1:11" s="15" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B34" s="16"/>
+      <c r="C34" s="16" t="s">
         <v>329</v>
       </c>
-      <c r="D31" s="30" t="s">
+      <c r="D34" s="15" t="s">
         <v>330</v>
       </c>
-      <c r="E31" s="30" t="s">
+      <c r="E34" s="15" t="s">
         <v>335</v>
       </c>
-      <c r="F31" s="30" t="s">
+      <c r="F34" s="15" t="s">
         <v>169</v>
       </c>
-      <c r="G31" s="30" t="s">
+      <c r="G34" s="15" t="s">
         <v>174</v>
       </c>
-      <c r="I31" s="30" t="s">
+      <c r="I34" s="15" t="s">
         <v>437</v>
       </c>
-      <c r="J31" s="34" t="s">
+      <c r="J34" s="16" t="s">
         <v>444</v>
       </c>
     </row>
-    <row r="32" spans="1:11" s="30" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="C32" s="32" t="s">
+    <row r="35" spans="1:11" s="15" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B35" s="16"/>
+      <c r="C35" s="16" t="s">
         <v>329</v>
       </c>
-      <c r="D32" s="30" t="s">
+      <c r="D35" s="15" t="s">
         <v>331</v>
       </c>
-      <c r="E32" s="30" t="s">
+      <c r="E35" s="15" t="s">
         <v>336</v>
       </c>
-      <c r="F32" s="30" t="s">
+      <c r="F35" s="15" t="s">
         <v>170</v>
       </c>
-      <c r="G32" s="30" t="s">
+      <c r="G35" s="15" t="s">
         <v>170</v>
       </c>
-      <c r="I32" s="30" t="s">
+      <c r="I35" s="15" t="s">
         <v>438</v>
       </c>
-      <c r="J32" s="34" t="s">
+      <c r="J35" s="16" t="s">
         <v>445</v>
       </c>
-      <c r="K32" s="34"/>
-    </row>
-    <row r="33" spans="1:11" s="30" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="C33" s="32" t="s">
+      <c r="K35" s="16"/>
+    </row>
+    <row r="36" spans="1:11" s="15" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B36" s="16"/>
+      <c r="C36" s="16" t="s">
         <v>329</v>
       </c>
-      <c r="D33" s="30" t="s">
+      <c r="D36" s="15" t="s">
         <v>332</v>
       </c>
-      <c r="E33" s="30" t="s">
+      <c r="E36" s="15" t="s">
         <v>337</v>
       </c>
-      <c r="F33" s="30" t="s">
+      <c r="F36" s="15" t="s">
         <v>171</v>
       </c>
-      <c r="G33" s="30" t="s">
+      <c r="G36" s="15" t="s">
         <v>175</v>
       </c>
-      <c r="I33" s="30" t="s">
+      <c r="I36" s="15" t="s">
         <v>439</v>
       </c>
-      <c r="J33" s="34" t="s">
+      <c r="J36" s="16" t="s">
         <v>446</v>
       </c>
-      <c r="K33" s="34"/>
-    </row>
-    <row r="34" spans="1:11" s="30" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="C34" s="32" t="s">
+      <c r="K36" s="16"/>
+    </row>
+    <row r="37" spans="1:11" s="15" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B37" s="16"/>
+      <c r="C37" s="16" t="s">
         <v>329</v>
       </c>
-      <c r="D34" s="30" t="s">
+      <c r="D37" s="15" t="s">
         <v>333</v>
       </c>
-      <c r="E34" s="30" t="s">
+      <c r="E37" s="15" t="s">
         <v>338</v>
       </c>
-      <c r="F34" s="30" t="s">
+      <c r="F37" s="15" t="s">
         <v>172</v>
       </c>
-      <c r="G34" s="30" t="s">
+      <c r="G37" s="15" t="s">
         <v>176</v>
       </c>
-      <c r="I34" s="30" t="s">
+      <c r="I37" s="15" t="s">
         <v>440</v>
       </c>
-      <c r="J34" s="34" t="s">
+      <c r="J37" s="16" t="s">
         <v>448</v>
       </c>
-      <c r="K34" s="34"/>
-    </row>
-    <row r="35" spans="1:11" s="30" customFormat="1" ht="31" x14ac:dyDescent="0.35">
-      <c r="C35" s="32" t="s">
+      <c r="K37" s="16"/>
+    </row>
+    <row r="38" spans="1:11" s="15" customFormat="1" ht="31" x14ac:dyDescent="0.35">
+      <c r="B38" s="16"/>
+      <c r="C38" s="16" t="s">
         <v>329</v>
       </c>
-      <c r="D35" s="30" t="s">
+      <c r="D38" s="15" t="s">
         <v>339</v>
       </c>
-      <c r="E35" s="30" t="s">
+      <c r="E38" s="15" t="s">
         <v>340</v>
       </c>
-      <c r="F35" s="30" t="s">
+      <c r="F38" s="15" t="s">
         <v>177</v>
       </c>
-      <c r="G35" s="30" t="s">
+      <c r="G38" s="15" t="s">
         <v>178</v>
       </c>
-      <c r="I35" s="30" t="s">
+      <c r="I38" s="15" t="s">
         <v>441</v>
       </c>
-      <c r="J35" s="34" t="s">
+      <c r="J38" s="16" t="s">
         <v>447</v>
       </c>
-      <c r="K35" s="34"/>
-    </row>
-    <row r="36" spans="1:11" s="30" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="C36" s="32" t="s">
+      <c r="K38" s="16"/>
+    </row>
+    <row r="39" spans="1:11" s="15" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B39" s="16"/>
+      <c r="C39" s="16" t="s">
         <v>329</v>
       </c>
-      <c r="D36" s="30" t="s">
+      <c r="D39" s="15" t="s">
         <v>334</v>
       </c>
-      <c r="E36" s="30" t="s">
+      <c r="E39" s="15" t="s">
         <v>341</v>
       </c>
-      <c r="F36" s="30" t="s">
+      <c r="F39" s="15" t="s">
         <v>173</v>
       </c>
-      <c r="G36" s="30" t="s">
+      <c r="G39" s="15" t="s">
         <v>173</v>
       </c>
-      <c r="I36" s="30" t="s">
+      <c r="I39" s="15" t="s">
         <v>442</v>
       </c>
-      <c r="J36" s="34" t="s">
+      <c r="J39" s="16" t="s">
         <v>449</v>
       </c>
-      <c r="K36" s="34"/>
-    </row>
-    <row r="37" spans="1:11" s="30" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="C37" s="32" t="s">
+      <c r="K39" s="16"/>
+    </row>
+    <row r="40" spans="1:11" s="15" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B40" s="16"/>
+      <c r="C40" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="E37" s="30" t="s">
+      <c r="E40" s="15" t="s">
         <v>429</v>
       </c>
-      <c r="F37" s="30" t="s">
+      <c r="F40" s="15" t="s">
         <v>85</v>
       </c>
-      <c r="G37" s="30" t="s">
+      <c r="G40" s="15" t="s">
         <v>91</v>
       </c>
-      <c r="I37" s="30" t="s">
+      <c r="I40" s="15" t="s">
         <v>443</v>
       </c>
-      <c r="J37" s="30" t="s">
+      <c r="J40" s="15" t="s">
         <v>431</v>
       </c>
-      <c r="K37" s="34"/>
-    </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A38" t="s">
+      <c r="K40" s="16"/>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="39" spans="1:11" s="30" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="C39" s="32" t="s">
+    <row r="42" spans="1:11" s="15" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B42" s="16"/>
+      <c r="C42" s="16" t="s">
         <v>397</v>
       </c>
-      <c r="F39" s="30" t="s">
+      <c r="F42" s="15" t="s">
         <v>432</v>
       </c>
-      <c r="G39" s="30" t="s">
+      <c r="G42" s="15" t="s">
         <v>433</v>
       </c>
-      <c r="I39" s="30" t="s">
+      <c r="I42" s="15" t="s">
         <v>424</v>
       </c>
-      <c r="J39" s="30" t="s">
+      <c r="J42" s="15" t="s">
         <v>430</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A40" t="s">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
         <v>450</v>
       </c>
     </row>
@@ -2934,7 +2951,60 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E4924F5-D4E0-4A82-97E5-002AF42E652B}">
+  <dimension ref="A1:C5"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" t="s">
+        <v>481</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:E105"/>
   <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -2959,7 +3029,7 @@
       <c r="D1" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="18" t="s">
+      <c r="E1" s="1" t="s">
         <v>346</v>
       </c>
     </row>
@@ -2976,7 +3046,7 @@
       <c r="D2" t="s">
         <v>89</v>
       </c>
-      <c r="E2" s="17" t="s">
+      <c r="E2" t="s">
         <v>348</v>
       </c>
     </row>
@@ -2993,7 +3063,7 @@
       <c r="D3" t="s">
         <v>90</v>
       </c>
-      <c r="E3" s="17" t="s">
+      <c r="E3" t="s">
         <v>349</v>
       </c>
     </row>
@@ -3010,7 +3080,7 @@
       <c r="D4" t="s">
         <v>91</v>
       </c>
-      <c r="E4" s="17" t="s">
+      <c r="E4" t="s">
         <v>350</v>
       </c>
     </row>
@@ -3027,7 +3097,7 @@
       <c r="D6" t="s">
         <v>153</v>
       </c>
-      <c r="E6" s="19" t="s">
+      <c r="E6" s="1" t="s">
         <v>351</v>
       </c>
     </row>
@@ -3044,7 +3114,7 @@
       <c r="D7" t="s">
         <v>154</v>
       </c>
-      <c r="E7" s="17" t="s">
+      <c r="E7" t="s">
         <v>352</v>
       </c>
     </row>
@@ -3061,7 +3131,7 @@
       <c r="D8" t="s">
         <v>155</v>
       </c>
-      <c r="E8" s="17" t="s">
+      <c r="E8" t="s">
         <v>353</v>
       </c>
     </row>
@@ -3069,16 +3139,16 @@
       <c r="A10" t="s">
         <v>94</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="8" t="s">
         <v>97</v>
       </c>
       <c r="C10" t="s">
         <v>108</v>
       </c>
-      <c r="D10" s="12" t="s">
+      <c r="D10" s="10" t="s">
         <v>113</v>
       </c>
-      <c r="E10" s="17" t="s">
+      <c r="E10" t="s">
         <v>354</v>
       </c>
     </row>
@@ -3086,16 +3156,16 @@
       <c r="A11" t="s">
         <v>94</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="8" t="s">
         <v>95</v>
       </c>
       <c r="C11" t="s">
         <v>104</v>
       </c>
-      <c r="D11" s="11" t="s">
+      <c r="D11" s="9" t="s">
         <v>114</v>
       </c>
-      <c r="E11" s="17" t="s">
+      <c r="E11" t="s">
         <v>355</v>
       </c>
     </row>
@@ -3103,16 +3173,16 @@
       <c r="A12" t="s">
         <v>94</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="B12" s="8" t="s">
         <v>103</v>
       </c>
       <c r="C12" t="s">
         <v>112</v>
       </c>
-      <c r="D12" s="12" t="s">
+      <c r="D12" s="10" t="s">
         <v>115</v>
       </c>
-      <c r="E12" s="17" t="s">
+      <c r="E12" t="s">
         <v>356</v>
       </c>
     </row>
@@ -3120,16 +3190,16 @@
       <c r="A13" t="s">
         <v>94</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="8" t="s">
         <v>96</v>
       </c>
       <c r="C13" t="s">
         <v>107</v>
       </c>
-      <c r="D13" s="13" t="s">
+      <c r="D13" s="11" t="s">
         <v>116</v>
       </c>
-      <c r="E13" s="17" t="s">
+      <c r="E13" t="s">
         <v>357</v>
       </c>
     </row>
@@ -3137,16 +3207,16 @@
       <c r="A14" t="s">
         <v>94</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="B14" s="8" t="s">
         <v>100</v>
       </c>
       <c r="C14" t="s">
         <v>111</v>
       </c>
-      <c r="D14" s="12" t="s">
+      <c r="D14" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="E14" s="19" t="s">
+      <c r="E14" s="1" t="s">
         <v>358</v>
       </c>
     </row>
@@ -3154,16 +3224,16 @@
       <c r="A15" t="s">
         <v>94</v>
       </c>
-      <c r="B15" s="10" t="s">
+      <c r="B15" s="8" t="s">
         <v>102</v>
       </c>
       <c r="C15" t="s">
         <v>106</v>
       </c>
-      <c r="D15" s="12" t="s">
+      <c r="D15" s="10" t="s">
         <v>118</v>
       </c>
-      <c r="E15" s="17" t="s">
+      <c r="E15" t="s">
         <v>359</v>
       </c>
     </row>
@@ -3171,16 +3241,16 @@
       <c r="A16" t="s">
         <v>94</v>
       </c>
-      <c r="B16" s="10" t="s">
+      <c r="B16" s="8" t="s">
         <v>99</v>
       </c>
       <c r="C16" t="s">
         <v>110</v>
       </c>
-      <c r="D16" s="12" t="s">
+      <c r="D16" s="10" t="s">
         <v>119</v>
       </c>
-      <c r="E16" s="17" t="s">
+      <c r="E16" t="s">
         <v>360</v>
       </c>
     </row>
@@ -3188,16 +3258,16 @@
       <c r="A17" t="s">
         <v>94</v>
       </c>
-      <c r="B17" s="10" t="s">
+      <c r="B17" s="8" t="s">
         <v>98</v>
       </c>
       <c r="C17" t="s">
         <v>109</v>
       </c>
-      <c r="D17" s="12" t="s">
+      <c r="D17" s="10" t="s">
         <v>120</v>
       </c>
-      <c r="E17" s="17" t="s">
+      <c r="E17" t="s">
         <v>361</v>
       </c>
     </row>
@@ -3205,16 +3275,16 @@
       <c r="A18" t="s">
         <v>94</v>
       </c>
-      <c r="B18" s="10" t="s">
+      <c r="B18" s="8" t="s">
         <v>101</v>
       </c>
       <c r="C18" t="s">
         <v>105</v>
       </c>
-      <c r="D18" s="12" t="s">
+      <c r="D18" s="10" t="s">
         <v>121</v>
       </c>
-      <c r="E18" s="17" t="s">
+      <c r="E18" t="s">
         <v>105</v>
       </c>
     </row>
@@ -3222,16 +3292,16 @@
       <c r="A19" t="s">
         <v>94</v>
       </c>
-      <c r="B19" s="15" t="s">
+      <c r="B19" s="13" t="s">
         <v>147</v>
       </c>
       <c r="C19" t="s">
         <v>148</v>
       </c>
-      <c r="D19" s="16" t="s">
+      <c r="D19" s="14" t="s">
         <v>156</v>
       </c>
-      <c r="E19" s="17" t="s">
+      <c r="E19" t="s">
         <v>362</v>
       </c>
     </row>
@@ -3239,16 +3309,16 @@
       <c r="A20" t="s">
         <v>94</v>
       </c>
-      <c r="B20" s="15" t="s">
+      <c r="B20" s="13" t="s">
         <v>149</v>
       </c>
       <c r="C20" t="s">
         <v>150</v>
       </c>
-      <c r="D20" s="16" t="s">
+      <c r="D20" s="14" t="s">
         <v>157</v>
       </c>
-      <c r="E20" s="19" t="s">
+      <c r="E20" s="1" t="s">
         <v>363</v>
       </c>
     </row>
@@ -3256,16 +3326,16 @@
       <c r="A21" t="s">
         <v>94</v>
       </c>
-      <c r="B21" s="15" t="s">
+      <c r="B21" s="13" t="s">
         <v>151</v>
       </c>
       <c r="C21" t="s">
         <v>152</v>
       </c>
-      <c r="D21" s="16" t="s">
+      <c r="D21" s="14" t="s">
         <v>158</v>
       </c>
-      <c r="E21" s="17" t="s">
+      <c r="E21" t="s">
         <v>364</v>
       </c>
     </row>
@@ -3273,226 +3343,209 @@
       <c r="A23" t="s">
         <v>126</v>
       </c>
-      <c r="B23" s="15" t="s">
+      <c r="B23" s="13" t="s">
         <v>163</v>
       </c>
-      <c r="C23" s="28" t="s">
+      <c r="C23" t="s">
         <v>169</v>
       </c>
-      <c r="D23" s="9" t="s">
+      <c r="D23" s="1" t="s">
         <v>174</v>
       </c>
-      <c r="E23" s="17"/>
-    </row>
-    <row r="24" spans="1:5" s="28" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="28" t="s">
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A24" t="s">
         <v>126</v>
       </c>
-      <c r="B24" s="15" t="s">
+      <c r="B24" s="13" t="s">
         <v>404</v>
       </c>
-      <c r="C24" s="28" t="s">
+      <c r="C24" t="s">
         <v>401</v>
       </c>
-      <c r="D24" s="9" t="s">
+      <c r="D24" s="1" t="s">
         <v>414</v>
       </c>
-      <c r="E24" s="29"/>
-    </row>
-    <row r="25" spans="1:5" s="28" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="28" t="s">
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A25" t="s">
         <v>126</v>
       </c>
-      <c r="B25" s="15" t="s">
+      <c r="B25" s="13" t="s">
         <v>167</v>
       </c>
-      <c r="C25" s="28" t="s">
+      <c r="C25" t="s">
         <v>177</v>
       </c>
-      <c r="D25" s="9" t="s">
+      <c r="D25" s="1" t="s">
         <v>178</v>
       </c>
-      <c r="E25" s="29"/>
-    </row>
-    <row r="26" spans="1:5" s="28" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="28" t="s">
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A26" t="s">
         <v>126</v>
       </c>
-      <c r="B26" s="15" t="s">
+      <c r="B26" s="13" t="s">
         <v>166</v>
       </c>
-      <c r="C26" s="28" t="s">
+      <c r="C26" t="s">
         <v>402</v>
       </c>
-      <c r="D26" s="14" t="s">
+      <c r="D26" s="12" t="s">
         <v>415</v>
       </c>
-      <c r="E26" s="29"/>
-    </row>
-    <row r="27" spans="1:5" s="28" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="28" t="s">
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A27" t="s">
         <v>126</v>
       </c>
-      <c r="B27" s="15" t="s">
+      <c r="B27" s="13" t="s">
         <v>168</v>
       </c>
-      <c r="C27" s="28" t="s">
+      <c r="C27" t="s">
         <v>173</v>
       </c>
-      <c r="D27" s="28" t="s">
+      <c r="D27" t="s">
         <v>173</v>
       </c>
-      <c r="E27" s="29"/>
-    </row>
-    <row r="28" spans="1:5" s="28" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="28" t="s">
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A28" t="s">
         <v>126</v>
       </c>
-      <c r="B28" s="15" t="s">
+      <c r="B28" s="13" t="s">
         <v>405</v>
       </c>
-      <c r="C28" s="28" t="s">
+      <c r="C28" t="s">
         <v>403</v>
       </c>
-      <c r="D28" s="9" t="s">
+      <c r="D28" s="1" t="s">
         <v>416</v>
       </c>
-      <c r="E28" s="29"/>
-    </row>
-    <row r="29" spans="1:5" s="28" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="28" t="s">
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A29" t="s">
         <v>126</v>
       </c>
-      <c r="B29" s="15" t="s">
+      <c r="B29" s="13" t="s">
         <v>88</v>
       </c>
-      <c r="C29" s="28" t="s">
+      <c r="C29" t="s">
         <v>85</v>
       </c>
-      <c r="D29" s="9" t="s">
+      <c r="D29" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="E29" s="29"/>
-    </row>
-    <row r="30" spans="1:5" s="28" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="B30" s="15"/>
-      <c r="D30" s="9"/>
-      <c r="E30" s="29"/>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="B30" s="13"/>
+      <c r="D30" s="1"/>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>129</v>
       </c>
-      <c r="B32" s="15" t="s">
+      <c r="B32" s="13" t="s">
         <v>407</v>
       </c>
-      <c r="C32" s="35" t="s">
+      <c r="C32" s="18" t="s">
         <v>391</v>
       </c>
       <c r="D32" t="s">
         <v>417</v>
       </c>
-      <c r="E32" s="17"/>
-    </row>
-    <row r="33" spans="1:5" ht="31" x14ac:dyDescent="0.35">
+    </row>
+    <row r="33" spans="1:4" ht="31" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>129</v>
       </c>
-      <c r="B33" s="15" t="s">
+      <c r="B33" s="13" t="s">
         <v>410</v>
       </c>
-      <c r="C33" s="35" t="s">
+      <c r="C33" s="18" t="s">
         <v>406</v>
       </c>
-      <c r="D33" s="9" t="s">
+      <c r="D33" s="1" t="s">
         <v>418</v>
       </c>
-      <c r="E33" s="17"/>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>129</v>
       </c>
-      <c r="B34" s="15" t="s">
+      <c r="B34" s="13" t="s">
         <v>411</v>
       </c>
-      <c r="C34" s="35" t="s">
+      <c r="C34" s="18" t="s">
         <v>392</v>
       </c>
-      <c r="D34" s="9" t="s">
+      <c r="D34" s="1" t="s">
         <v>419</v>
       </c>
-      <c r="E34" s="17"/>
-    </row>
-    <row r="35" spans="1:5" s="28" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="28" t="s">
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
         <v>129</v>
       </c>
-      <c r="B35" s="15" t="s">
+      <c r="B35" s="13" t="s">
         <v>412</v>
       </c>
-      <c r="C35" s="35" t="s">
+      <c r="C35" s="18" t="s">
         <v>393</v>
       </c>
-      <c r="D35" s="9" t="s">
+      <c r="D35" s="1" t="s">
         <v>420</v>
       </c>
-      <c r="E35" s="29"/>
-    </row>
-    <row r="36" spans="1:5" s="28" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="28" t="s">
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
         <v>129</v>
       </c>
-      <c r="B36" s="15" t="s">
+      <c r="B36" s="13" t="s">
         <v>413</v>
       </c>
-      <c r="C36" s="35" t="s">
+      <c r="C36" s="18" t="s">
         <v>394</v>
       </c>
-      <c r="D36" s="9" t="s">
+      <c r="D36" s="1" t="s">
         <v>421</v>
       </c>
-      <c r="E36" s="29"/>
-    </row>
-    <row r="37" spans="1:5" s="28" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="28" t="s">
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
         <v>129</v>
       </c>
-      <c r="B37" s="15" t="s">
+      <c r="B37" s="13" t="s">
         <v>408</v>
       </c>
-      <c r="C37" s="35" t="s">
+      <c r="C37" s="18" t="s">
         <v>395</v>
       </c>
-      <c r="D37" s="9" t="s">
+      <c r="D37" s="1" t="s">
         <v>422</v>
       </c>
-      <c r="E37" s="29"/>
-    </row>
-    <row r="38" spans="1:5" s="28" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A38" s="28" t="s">
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
         <v>129</v>
       </c>
-      <c r="B38" s="15" t="s">
+      <c r="B38" s="13" t="s">
         <v>409</v>
       </c>
-      <c r="C38" s="35" t="s">
+      <c r="C38" s="18" t="s">
         <v>396</v>
       </c>
-      <c r="D38" s="9" t="s">
+      <c r="D38" s="1" t="s">
         <v>423</v>
       </c>
-      <c r="E38" s="29"/>
-    </row>
-    <row r="39" spans="1:5" s="28" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="D39" s="9"/>
-      <c r="E39" s="29"/>
-    </row>
-    <row r="40" spans="1:5" s="28" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="D40" s="9"/>
-      <c r="E40" s="29"/>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="D39" s="1"/>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="D40" s="1"/>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>328</v>
       </c>
@@ -3506,7 +3559,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>328</v>
       </c>
@@ -3520,7 +3573,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>328</v>
       </c>
@@ -3534,7 +3587,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>328</v>
       </c>
@@ -3548,7 +3601,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>328</v>
       </c>
@@ -3562,7 +3615,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>328</v>
       </c>
@@ -3576,7 +3629,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>330</v>
       </c>
@@ -4315,7 +4368,7 @@
       <c r="C105" t="s">
         <v>342</v>
       </c>
-      <c r="D105" s="9" t="s">
+      <c r="D105" s="1" t="s">
         <v>344</v>
       </c>
     </row>
@@ -4325,9 +4378,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H2"/>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+  <dimension ref="A1:H4"/>
   <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="21.5" customWidth="1"/>
@@ -4342,28 +4395,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="G1" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="H1" s="4" t="s">
         <v>31</v>
       </c>
     </row>
@@ -4392,6 +4445,35 @@
       <c r="H2" t="s">
         <v>37</v>
       </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>478</v>
+      </c>
+      <c r="B3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" t="s">
+        <v>34</v>
+      </c>
+      <c r="D3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E3" s="19" t="s">
+        <v>476</v>
+      </c>
+      <c r="F3" t="s">
+        <v>477</v>
+      </c>
+      <c r="G3" t="s">
+        <v>37</v>
+      </c>
+      <c r="H3" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="E4" s="19"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.51180555555555496" footer="0.51180555555555496"/>
@@ -4404,16 +4486,15 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:H9"/>
   <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
     <col min="2" max="2" width="8.5" customWidth="1"/>
     <col min="3" max="3" width="19.83203125" customWidth="1"/>
-    <col min="4" max="4" width="17.08203125" customWidth="1"/>
-    <col min="5" max="5" width="17.08203125" style="20" customWidth="1"/>
+    <col min="4" max="5" width="17.08203125" customWidth="1"/>
     <col min="6" max="6" width="20.33203125" customWidth="1"/>
     <col min="7" max="7" width="20.75" customWidth="1"/>
     <col min="8" max="8" width="22" customWidth="1"/>
@@ -4433,7 +4514,7 @@
       <c r="D1" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="24" t="s">
+      <c r="E1" t="s">
         <v>346</v>
       </c>
       <c r="F1" t="s">
@@ -4442,7 +4523,7 @@
       <c r="G1" t="s">
         <v>41</v>
       </c>
-      <c r="H1" s="27" t="s">
+      <c r="H1" t="s">
         <v>372</v>
       </c>
     </row>
@@ -4453,8 +4534,6 @@
       <c r="B2" t="s">
         <v>76</v>
       </c>
-      <c r="E2" s="23"/>
-      <c r="H2" s="26"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
@@ -4463,8 +4542,6 @@
       <c r="B3" t="s">
         <v>76</v>
       </c>
-      <c r="E3" s="23"/>
-      <c r="H3" s="26"/>
     </row>
     <row r="4" spans="1:8" ht="31" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
@@ -4476,43 +4553,37 @@
       <c r="D4" t="s">
         <v>46</v>
       </c>
-      <c r="E4" s="25" t="s">
+      <c r="E4" s="1" t="s">
         <v>371</v>
       </c>
-      <c r="H4" s="26"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="B5" s="6">
+      <c r="B5" s="5">
         <v>20170804</v>
       </c>
-      <c r="E5" s="23"/>
-      <c r="H5" s="26"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>48</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" t="s">
         <v>19</v>
       </c>
-      <c r="E6" s="23"/>
-      <c r="H6" s="26"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>49</v>
       </c>
-      <c r="E7" s="23"/>
       <c r="F7" t="s">
         <v>50</v>
       </c>
       <c r="G7" t="s">
         <v>51</v>
       </c>
-      <c r="H7" s="27" t="s">
+      <c r="H7" t="s">
         <v>373</v>
       </c>
     </row>
@@ -4520,14 +4591,13 @@
       <c r="A8" t="s">
         <v>52</v>
       </c>
-      <c r="E8" s="23"/>
       <c r="F8" t="s">
         <v>53</v>
       </c>
       <c r="G8" t="s">
         <v>54</v>
       </c>
-      <c r="H8" s="27" t="s">
+      <c r="H8" t="s">
         <v>374</v>
       </c>
     </row>
@@ -4535,14 +4605,13 @@
       <c r="A9" t="s">
         <v>378</v>
       </c>
-      <c r="E9" s="23"/>
-      <c r="F9" s="29" t="s">
+      <c r="F9" t="s">
         <v>377</v>
       </c>
-      <c r="G9" s="28" t="s">
+      <c r="G9" t="s">
         <v>376</v>
       </c>
-      <c r="H9" s="27" t="s">
+      <c r="H9" t="s">
         <v>375</v>
       </c>
     </row>
@@ -4552,8 +4621,8 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:E8"/>
   <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -4582,121 +4651,121 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="D2" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="E2" s="6" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="6" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="E4" s="6" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A5" s="3" t="s">
+      <c r="A5" t="s">
         <v>58</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" t="s">
         <v>64</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" t="s">
         <v>65</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" t="s">
         <v>66</v>
       </c>
-      <c r="E5" s="8" t="s">
+      <c r="E5" s="7" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A6" s="3" t="s">
+      <c r="A6" t="s">
         <v>58</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" t="s">
         <v>64</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" t="s">
         <v>68</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="8" t="s">
+      <c r="E6" s="7" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A7" s="3" t="s">
+      <c r="A7" t="s">
         <v>70</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" t="s">
         <v>59</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" t="s">
         <v>71</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="D7" t="s">
         <v>12</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="E7" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A8" s="3" t="s">
+      <c r="A8" t="s">
         <v>73</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" t="s">
         <v>59</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" t="s">
         <v>74</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="D8" t="s">
         <v>12</v>
       </c>
-      <c r="E8" s="3" t="s">
+      <c r="E8" t="s">
         <v>75</v>
       </c>
     </row>

</xml_diff>